<commit_message>
x1514 Change sample.section (and all related fields) to be a string
Sample section (formerly an int) is now a positive int
plus optional letters.
i.e. [1-9][0-9]*[a-z]*
Everywhere it was referenced as an int has to be changed to a string.
Also put it in lower case for consistency.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/section_reg.xlsx
+++ b/src/test/resources/testdata/section_reg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dr6/Code/stan/core/src/test/resources/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C6226E-3BFC-724A-9B27-D88CB741ADAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18274E9A-A1D2-5446-B6AF-871064AFA8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2600" yWindow="1000" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2600" yWindow="900" windowWidth="27640" windowHeight="16940" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="57">
   <si>
     <r>
       <t xml:space="preserve">SGP number
@@ -413,6 +413,9 @@
   </si>
   <si>
     <t>Homo sapiens (Human)</t>
+  </si>
+  <si>
+    <t>13a</t>
   </si>
 </sst>
 </file>
@@ -1180,8 +1183,8 @@
       <c r="R4" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="S4" s="17">
-        <v>12</v>
+      <c r="S4" s="17" t="s">
+        <v>56</v>
       </c>
       <c r="T4" s="17" t="s">
         <v>36</v>

</xml_diff>